<commit_message>
feat: re-include paper 225 (Lalos 2024) as employee sample and extract 8 effect sizes
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/203_207_208_225.xlsx
+++ b/03_Coding_Sheets/203_207_208_225.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX38"/>
+  <dimension ref="A1:AX45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5393,12 +5393,1066 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = include</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>2 = Non-employee samples</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V38" t="n">
+        <v>143</v>
+      </c>
+      <c r="W38" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X38" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA38" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH38" t="n">
+        <v>9</v>
+      </c>
+      <c r="AI38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK38" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>Pearce et al., 1991</t>
+        </is>
+      </c>
+      <c r="AN38" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 48-49] "interaction was measured using an established interdependence scale (Pearce et al., 1991) due to its reliability and validity of measuring employee-perceived, self-report task interdependence." Original 10-item scale; 1 item removed to increase alpha from 0.691 to 0.707, yielding 9 final items. Each item on 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). Adapted to freelancer/contracting organization context.</t>
+        </is>
+      </c>
+      <c r="AO38" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP38" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ38" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR38" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS38" t="inlineStr">
+        <is>
+          <t>Task Interdependence</t>
+        </is>
+      </c>
+      <c r="AT38" t="n">
+        <v>3.717</v>
+      </c>
+      <c r="AU38" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="AV38" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="AW38" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="AX38" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: Task Interdependence, Col: Boundary Spanning, Raw: 0.183*</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>225</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V39" t="n">
+        <v>143</v>
+      </c>
+      <c r="W39" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X39" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA39" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH39" t="n">
+        <v>6</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK39" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>Hinkin et al. (1989)</t>
+        </is>
+      </c>
+      <c r="AN39" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 49-50] "The 4-item Hinkin et al. (1989) expert power scale was adapted from the seminal work of French et al. (1959)." Original 4-item scale augmented with 2 additional items after pilot study to increase alpha from 0.745 to 0.800. Items operationalized to reflect freelancer self-perspective of expert influence. All items on 5-point Likert from Strongly Disagree (1) to Strongly Agree (5).</t>
+        </is>
+      </c>
+      <c r="AO39" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP39" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR39" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>Expert Power</t>
+        </is>
+      </c>
+      <c r="AT39" t="n">
+        <v>4.307</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="AV39" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AW39" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="AX39" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: Expert Power, Col: Boundary Spanning, Raw: 0.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>225</v>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V40" t="n">
+        <v>143</v>
+      </c>
+      <c r="W40" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X40" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA40" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG40" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH40" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI40" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ40" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK40" t="inlineStr">
+        <is>
+          <t>4 = Objective</t>
+        </is>
+      </c>
+      <c r="AL40" t="inlineStr">
+        <is>
+          <t>Secondary data extracted from Upwork profiles and resumes; not a survey-administered scale.</t>
+        </is>
+      </c>
+      <c r="AN40" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51] "Human capital measures primarily rely on the skilled freelancer's profile and what others in the organization see. college degree and certifications completed were collected from the profile of each respondent to objectively gauge relative differences in human capital across individual participants." Education level operationalized as ordinal: low (no education/associate degree=1), medium (bachelor's=2), high (master's/PhD=3). Working experience (years) also collected. M=12.028 SD=9.795 reflects working experience operationalization.</t>
+        </is>
+      </c>
+      <c r="AO40" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP40" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ40" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR40" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS40" t="inlineStr">
+        <is>
+          <t>Human Capital</t>
+        </is>
+      </c>
+      <c r="AT40" t="n">
+        <v>12.028</v>
+      </c>
+      <c r="AU40" t="n">
+        <v>9.795</v>
+      </c>
+      <c r="AV40" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW40" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="AX40" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: Human Capital, Col: Boundary Spanning, Raw: 0.102</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>225</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V41" t="n">
+        <v>143</v>
+      </c>
+      <c r="W41" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X41" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA41" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH41" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ41" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK41" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>Hinkin &amp; Schriesheim, 1989</t>
+        </is>
+      </c>
+      <c r="AN41" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 50-51] "Specifically, the 4-item referent power scale (Hinkin &amp; Schriesheim, 1989) was applied as a post hoc test." Items adapted for freelancer context. Self-perspective assessment of perceived referent power. All items on 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). M/SD not recoverable from PDF text extraction (Table 1 multi-column layout collision).</t>
+        </is>
+      </c>
+      <c r="AO41" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP41" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ41" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR41" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS41" t="inlineStr">
+        <is>
+          <t>Referent Power</t>
+        </is>
+      </c>
+      <c r="AT41" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU41" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV41" t="n">
+        <v>0.897</v>
+      </c>
+      <c r="AW41" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="AX41" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: Referent Power, Col: Boundary Spanning, Raw: 0.118</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>225</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V42" t="n">
+        <v>143</v>
+      </c>
+      <c r="W42" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X42" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA42" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH42" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ42" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK42" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM42" t="inlineStr">
+        <is>
+          <t>Soda et al., 2018</t>
+        </is>
+      </c>
+      <c r="AN42" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 50] "Collaboration was assessed using an established strategic orientation toward brokering scale (Soda et al., 2018)." Collaborate sub-scale only (arbitrage sub-scale excluded, alpha=0.295 unacceptable). Original 6-item collaborate sub-scale; 1 item removed to increase alpha from 0.779 to 0.824, yielding 5 final items. Table 3 (p. 119) renders 0.825. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5).</t>
+        </is>
+      </c>
+      <c r="AO42" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP42" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ42" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR42" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS42" t="inlineStr">
+        <is>
+          <t>Strategic Orientation - Collaboration</t>
+        </is>
+      </c>
+      <c r="AT42" t="n">
+        <v>3.527</v>
+      </c>
+      <c r="AU42" t="n">
+        <v>0.705</v>
+      </c>
+      <c r="AV42" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="AW42" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="AX42" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: Strategic Orientation - Collaboration, Col: Boundary Spanning, Raw: 0.268</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>225</v>
+      </c>
+      <c r="D43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V43" t="n">
+        <v>143</v>
+      </c>
+      <c r="W43" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X43" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA43" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK43" t="inlineStr">
+        <is>
+          <t>4 = Objective</t>
+        </is>
+      </c>
+      <c r="AL43" t="inlineStr">
+        <is>
+          <t>Upwork platform job success score — objective secondary data.</t>
+        </is>
+      </c>
+      <c r="AN43" t="inlineStr">
+        <is>
+          <t>Upwork platform job success rating (objective secondary data from freelancer profiles). Not a multi-item survey scale; no Cronbach alpha applicable. M/SD not recoverable from PDF text extraction (Table 1 multi-column layout collision).</t>
+        </is>
+      </c>
+      <c r="AO43" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP43" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ43" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR43" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS43" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="AT43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW43" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AX43" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: Rating, Col: Boundary Spanning, Raw: 0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>225</v>
+      </c>
+      <c r="D44" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V44" t="n">
+        <v>143</v>
+      </c>
+      <c r="W44" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X44" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA44" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>4 = Objective</t>
+        </is>
+      </c>
+      <c r="AL44" t="inlineStr">
+        <is>
+          <t>Binary work arrangement variable from Upwork profile data.</t>
+        </is>
+      </c>
+      <c r="AN44" t="inlineStr">
+        <is>
+          <t>Remote Work: binary indicator variable from secondary Upwork profile data (remote vs. non-remote work arrangement). Not a multi-item survey scale. M/SD not recoverable from PDF text extraction (Table 1 multi-column layout collision).</t>
+        </is>
+      </c>
+      <c r="AO44" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP44" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ44" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR44" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>Remote Work</t>
+        </is>
+      </c>
+      <c r="AT44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW44" t="n">
+        <v>-0.127</v>
+      </c>
+      <c r="AX44" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: Remote Work, Col: Boundary Spanning, Raw: -0.127</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>225</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V45" t="n">
+        <v>143</v>
+      </c>
+      <c r="W45" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X45" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA45" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH45" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>4 = Objective</t>
+        </is>
+      </c>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>Contract duration from Upwork profile data (hours/weeks).</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr">
+        <is>
+          <t>Contract Time: contract duration variable from secondary Upwork profile data. Not a multi-item survey scale. M/SD not recoverable from PDF text extraction (Table 1 multi-column layout collision).</t>
+        </is>
+      </c>
+      <c r="AO45" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP45" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>Contract Time</t>
+        </is>
+      </c>
+      <c r="AT45" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW45" t="n">
+        <v>-0.131</v>
+      </c>
+      <c r="AX45" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: Contract Time, Col: Boundary Spanning, Raw: -0.131</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Gender effect size row (ES#9) for Paper 225 in 203_207_208_225.xlsx
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/203_207_208_225.xlsx
+++ b/03_Coding_Sheets/203_207_208_225.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX45"/>
+  <dimension ref="A1:AX46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6453,6 +6453,135 @@
       <c r="AX45" t="inlineStr">
         <is>
           <t>Table 2 (p. 122), Row: Contract Time, Col: Boundary Spanning, Raw: -0.131</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>225</v>
+      </c>
+      <c r="D46" t="n">
+        <v>9</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V46" t="n">
+        <v>143</v>
+      </c>
+      <c r="W46" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="X46" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Skilled Digital Freelancers (Accountants and Software Engineers via Upwork)</t>
+        </is>
+      </c>
+      <c r="AA46" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>Ancona et al. (1992A)</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>[Methodology, p. 51-52] "Ancona et al. (1992A) developed a boundary spanning scale that aids in understanding boundary spanning at a micro level. The six scouting items from this scale were used for this study because they measure high-frequency communicators, expertise, and access to information, which are characteristics of skilled digital freelancers." Scouting sub-dimension only. Items adapted: network wording substituted for competing organization wording due to non-disclosure concerns. 5-point Likert from Strongly Disagree (1) to Strongly Agree (5). In-text alpha = 0.858; Table 3 (p. 119) renders 0.859.</t>
+        </is>
+      </c>
+      <c r="AH46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ46" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK46" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AN46" t="inlineStr">
+        <is>
+          <t>[Appendix F: Survey Instrument, p. 111] "2.) The gender you identify with is: a. Male b. Female c. Non-binary/third gender d. Prefer not to say" [Sample, p. 61] "Forty seven percent of participants identified as female (n = 66) and 53% as male (n = 77)."</t>
+        </is>
+      </c>
+      <c r="AO46" t="inlineStr">
+        <is>
+          <t>Boundary Spanning</t>
+        </is>
+      </c>
+      <c r="AP46" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AQ46" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AR46" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="AS46" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="AT46" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU46" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV46" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW46" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="AX46" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 122), Row: 8. Gender, Col: 1. Boundary Spanning, Raw: 0.066</t>
         </is>
       </c>
     </row>

</xml_diff>